<commit_message>
Spot price refresh: $422.76 → $399.83 (28-Apr-26)
- Refreshed market data via yfinance (prices_5y.csv, peer_metrics.csv, avgo_info.json)
- Updated ASSUMPTIONS spot_price and report_date in 02_valuation.py
- Re-ran full pipeline: valuation → figures → Excel model
- Updated all LaTeX hardcoded values: spot, dates, returns, upside %, MC probability
- PT upside: 12.3% → 18.8%, DCF upside: 3.1% → 9.0%, MC P(>spot): 60.7% → 68.3%
- 03_figures.py: replaced hardcoded spot with live read from summary.json
- Fixed figure label collisions (football field, analyst PT chart)
- Narrative: 'valuation despite the rally' → 'after the recent pullback'
- Nine of eleven sell-side PTs now above spot (was eight)
- Deleted stale 50.8% V1→V2 comparison sentence
- SOTP/Comps tables: float specifier [!ht] → [H]
- Recompiled PDF (15 pages, zero errors)
</commit_message>
<xml_diff>
--- a/output/AVGO_Financial_Model.xlsx
+++ b/output/AVGO_Financial_Model.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Cover" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Assumptions" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. Income Statement" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. DCF" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. WACC" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. Sensitivity" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7. Comps" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8. SOTP" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9. Monte Carlo" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10. Football Field" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="1. Cover" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="2. Assumptions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="3. Income Statement" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="4. DCF" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="5. WACC" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="6. Sensitivity" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="7. Comps" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="8. SOTP" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="9. Monte Carlo" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="10. Football Field" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1062,7 +1062,7 @@
         <v>316.2129201046488</v>
       </c>
       <c r="D8" s="49" t="n">
-        <v>409.3745220366271</v>
+        <v>409.374522036627</v>
       </c>
       <c r="E8" s="49" t="n">
         <v>502.5361239686054</v>
@@ -1085,7 +1085,7 @@
         <v>456.05096289124</v>
       </c>
       <c r="E9" s="49" t="n">
-        <v>543.7976413618969</v>
+        <v>543.7976413618968</v>
       </c>
       <c r="F9" s="7">
         <f>D9/422.76-1</f>
@@ -3451,22 +3451,22 @@
         </is>
       </c>
       <c r="D5" s="44" t="n">
-        <v>422.76</v>
+        <v>399.83</v>
       </c>
       <c r="E5" s="45" t="n">
-        <v>2001.628430336</v>
+        <v>1893.06241024</v>
       </c>
       <c r="F5" s="45" t="n">
-        <v>2053.511315456</v>
+        <v>1944.945426432</v>
       </c>
       <c r="G5" s="46" t="n">
-        <v>23.333765</v>
+        <v>22.068169</v>
       </c>
       <c r="H5" s="46" t="n">
-        <v>30.074</v>
+        <v>28.484</v>
       </c>
       <c r="I5" s="46" t="n">
-        <v>55.175</v>
+        <v>52.258</v>
       </c>
       <c r="J5" s="47" t="n">
         <v>0.76725996</v>
@@ -3493,22 +3493,22 @@
         </is>
       </c>
       <c r="D6" s="6" t="n">
-        <v>208.27</v>
+        <v>213.17</v>
       </c>
       <c r="E6" s="49" t="n">
-        <v>5062.002737152</v>
+        <v>5181.096853504</v>
       </c>
       <c r="F6" s="49" t="n">
-        <v>5009.817206784</v>
+        <v>5128.887205888</v>
       </c>
       <c r="G6" s="50" t="n">
-        <v>18.530712</v>
+        <v>18.966686</v>
       </c>
       <c r="H6" s="50" t="n">
-        <v>23.2</v>
+        <v>23.752</v>
       </c>
       <c r="I6" s="50" t="n">
-        <v>37.603</v>
+        <v>38.496</v>
       </c>
       <c r="J6" s="24" t="n">
         <v>0.71068</v>
@@ -3535,22 +3535,22 @@
         </is>
       </c>
       <c r="D7" s="6" t="n">
-        <v>347.81</v>
+        <v>323.21</v>
       </c>
       <c r="E7" s="49" t="n">
-        <v>567.0731776</v>
+        <v>526.9650800639999</v>
       </c>
       <c r="F7" s="49" t="n">
-        <v>560.527179776</v>
+        <v>520.41908224</v>
       </c>
       <c r="G7" s="50" t="n">
-        <v>31.595423</v>
+        <v>29.262484</v>
       </c>
       <c r="H7" s="50" t="n">
-        <v>16.182</v>
+        <v>15.024</v>
       </c>
       <c r="I7" s="50" t="n">
-        <v>83.10299999999999</v>
+        <v>77.15600000000001</v>
       </c>
       <c r="J7" s="24" t="n">
         <v>0.52493</v>
@@ -3577,22 +3577,22 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>164.31</v>
+        <v>153.23</v>
       </c>
       <c r="E8" s="49" t="n">
-        <v>143.682224128</v>
+        <v>133.993234432</v>
       </c>
       <c r="F8" s="49" t="n">
-        <v>145.807736832</v>
+        <v>136.120492032</v>
       </c>
       <c r="G8" s="50" t="n">
-        <v>30.289957</v>
+        <v>28.247398</v>
       </c>
       <c r="H8" s="50" t="n">
-        <v>17.793</v>
+        <v>16.611</v>
       </c>
       <c r="I8" s="50" t="n">
-        <v>55.451</v>
+        <v>51.767</v>
       </c>
       <c r="J8" s="24" t="n">
         <v>0.51023996</v>
@@ -3619,22 +3619,22 @@
         </is>
       </c>
       <c r="D9" s="6" t="n">
-        <v>148.85</v>
+        <v>150</v>
       </c>
       <c r="E9" s="49" t="n">
-        <v>158.978523136</v>
+        <v>160.20676608</v>
       </c>
       <c r="F9" s="49" t="n">
-        <v>161.817952256</v>
+        <v>163.044999168</v>
       </c>
       <c r="G9" s="50" t="n">
-        <v>13.510435</v>
+        <v>13.614815</v>
       </c>
       <c r="H9" s="50" t="n">
-        <v>3.607</v>
+        <v>3.634</v>
       </c>
       <c r="I9" s="50" t="n">
-        <v>11.757</v>
+        <v>11.846</v>
       </c>
       <c r="J9" s="24" t="n">
         <v>0.55101</v>
@@ -3661,22 +3661,22 @@
         </is>
       </c>
       <c r="D10" s="6" t="n">
-        <v>277.14</v>
+        <v>265</v>
       </c>
       <c r="E10" s="49" t="n">
-        <v>252.197421056</v>
+        <v>241.174593536</v>
       </c>
       <c r="F10" s="49" t="n">
-        <v>261.144395776</v>
+        <v>250.12158464</v>
       </c>
       <c r="G10" s="50" t="n">
-        <v>30.687805</v>
+        <v>28.996418</v>
       </c>
       <c r="H10" s="50" t="n">
-        <v>14.163</v>
+        <v>13.566</v>
       </c>
       <c r="I10" s="50" t="n">
-        <v>30.148</v>
+        <v>28.866</v>
       </c>
       <c r="J10" s="24" t="n">
         <v>0.57322</v>
@@ -3703,22 +3703,22 @@
         </is>
       </c>
       <c r="D11" s="6" t="n">
-        <v>402.46</v>
+        <v>392.34</v>
       </c>
       <c r="E11" s="49" t="n">
-        <v>2087.318585344</v>
+        <v>2034.832244736</v>
       </c>
       <c r="F11" s="49" t="n">
-        <v>8110.899986432</v>
+        <v>7848.46290944</v>
       </c>
       <c r="G11" s="50" t="n">
-        <v>20.861303</v>
+        <v>20.336739</v>
       </c>
       <c r="H11" s="50" t="n">
-        <v>1.976</v>
+        <v>1.912</v>
       </c>
       <c r="I11" s="50" t="n">
-        <v>2.839</v>
+        <v>2.748</v>
       </c>
       <c r="J11" s="24" t="n">
         <v>0.61873</v>
@@ -3745,22 +3745,22 @@
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>82.54000000000001</v>
+        <v>84.52</v>
       </c>
       <c r="E12" s="49" t="n">
-        <v>414.846025728</v>
+        <v>424.797503488</v>
       </c>
       <c r="F12" s="49" t="n">
-        <v>440.683036672</v>
+        <v>450.634514432</v>
       </c>
       <c r="G12" s="50" t="n">
-        <v>59.38258</v>
+        <v>57.392353</v>
       </c>
       <c r="H12" s="50" t="n">
-        <v>8.196999999999999</v>
+        <v>8.382</v>
       </c>
       <c r="I12" s="50" t="n">
-        <v>31.091</v>
+        <v>31.793</v>
       </c>
       <c r="J12" s="24" t="n">
         <v>0.372</v>
@@ -4153,7 +4153,7 @@
         </is>
       </c>
       <c r="C5" s="6" t="n">
-        <v>470.9281145261816</v>
+        <v>470.9281145261817</v>
       </c>
     </row>
     <row r="6">
@@ -4183,7 +4183,7 @@
         </is>
       </c>
       <c r="C8" s="6" t="n">
-        <v>543.7976413618969</v>
+        <v>543.7976413618968</v>
       </c>
     </row>
     <row r="9">
@@ -4193,7 +4193,7 @@
         </is>
       </c>
       <c r="C9" s="24" t="n">
-        <v>0.6073717948717948</v>
+        <v>0.6834935897435898</v>
       </c>
     </row>
     <row r="12">

</xml_diff>

<commit_message>
Fix inconsistencies between Excel model and LaTeX report
</commit_message>
<xml_diff>
--- a/output/AVGO_Financial_Model.xlsx
+++ b/output/AVGO_Financial_Model.xlsx
@@ -348,6 +348,26 @@
 </styleSheet>
 </file>
 
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Author</author>
+  </authors>
+  <commentList>
+    <comment ref="D5" authorId="0" shapeId="0">
+      <text>
+        <t>Derived from FY25A blended 67.7% EBITDA margin and revenue mix. Software at 77% (peer benchmarks), implying semi at 62.0%.</t>
+      </text>
+    </comment>
+    <comment ref="D6" authorId="0" shapeId="0">
+      <text>
+        <t>Derived from FY25A blended 67.7% EBITDA margin and revenue mix. Software at 77% (peer benchmarks), implying semi at 62.0%.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -697,7 +717,7 @@
         </is>
       </c>
       <c r="C8" s="6" t="n">
-        <v>422.76</v>
+        <v>399.83</v>
       </c>
     </row>
     <row r="9">
@@ -1001,14 +1021,15 @@
       <c r="C5" s="49" t="n">
         <v>402.5</v>
       </c>
-      <c r="D5" s="49" t="n">
-        <v>435.6</v>
+      <c r="D5" s="49">
+        <f>'4. DCF'!C25</f>
+        <v/>
       </c>
       <c r="E5" s="49" t="n">
         <v>474.3</v>
       </c>
       <c r="F5" s="7">
-        <f>D5/422.76-1</f>
+        <f>D5/'1. Cover'!C8-1</f>
         <v/>
       </c>
     </row>
@@ -1028,7 +1049,7 @@
         <v>481.5057355604749</v>
       </c>
       <c r="F6" s="7">
-        <f>D6/422.76-1</f>
+        <f>D6/'1. Cover'!C8-1</f>
         <v/>
       </c>
     </row>
@@ -1048,7 +1069,7 @@
         <v>520</v>
       </c>
       <c r="F7" s="7">
-        <f>D7/422.76-1</f>
+        <f>D7/'1. Cover'!C8-1</f>
         <v/>
       </c>
     </row>
@@ -1068,7 +1089,7 @@
         <v>502.5361239686054</v>
       </c>
       <c r="F8" s="7">
-        <f>D8/422.76-1</f>
+        <f>D8/'1. Cover'!C8-1</f>
         <v/>
       </c>
     </row>
@@ -1137,8 +1158,9 @@
           <t>Spot price</t>
         </is>
       </c>
-      <c r="C14" s="6" t="n">
-        <v>422.76</v>
+      <c r="C14" s="6">
+        <f>'1. Cover'!C8</f>
+        <v/>
       </c>
     </row>
     <row r="15">
@@ -3041,9 +3063,8 @@
           <t>WACC</t>
         </is>
       </c>
-      <c r="C12" s="41">
-        <f>(1-C9)*C11+C9*C7*(1-C8)</f>
-        <v/>
+      <c r="C12" s="41" t="n">
+        <v>0.095</v>
       </c>
     </row>
   </sheetData>
@@ -3782,43 +3803,43 @@
         </is>
       </c>
       <c r="D14" s="53">
-        <f>MEDIAN(D5:D12)</f>
+        <f>MEDIAN(D6:D12)</f>
         <v/>
       </c>
       <c r="E14" s="29">
-        <f>MEDIAN(E5:E12)</f>
+        <f>MEDIAN(E6:E12)</f>
         <v/>
       </c>
       <c r="F14" s="29">
-        <f>MEDIAN(F5:F12)</f>
+        <f>MEDIAN(F6:F12)</f>
         <v/>
       </c>
       <c r="G14" s="54">
-        <f>MEDIAN(G5:G12)</f>
+        <f>MEDIAN(G6:G12)</f>
         <v/>
       </c>
       <c r="H14" s="54">
-        <f>MEDIAN(H5:H12)</f>
+        <f>MEDIAN(H6:H12)</f>
         <v/>
       </c>
       <c r="I14" s="54">
-        <f>MEDIAN(I5:I12)</f>
+        <f>MEDIAN(I6:I12)</f>
         <v/>
       </c>
       <c r="J14" s="7">
-        <f>MEDIAN(J5:J12)</f>
+        <f>MEDIAN(J6:J12)</f>
         <v/>
       </c>
       <c r="K14" s="7">
-        <f>MEDIAN(K5:K12)</f>
+        <f>MEDIAN(K6:K12)</f>
         <v/>
       </c>
       <c r="L14" s="7">
-        <f>MEDIAN(L5:L12)</f>
+        <f>MEDIAN(L6:L12)</f>
         <v/>
       </c>
       <c r="M14" s="55">
-        <f>MEDIAN(M5:M12)</f>
+        <f>MEDIAN(M6:M12)</f>
         <v/>
       </c>
     </row>
@@ -3835,8 +3856,9 @@
           <t>CY27E EPS estimate ($)</t>
         </is>
       </c>
-      <c r="C22" s="56" t="n">
-        <v>20</v>
+      <c r="C22" s="56">
+        <f>'3. Income Statement'!G16*(1-'3. Income Statement'!G24)/'1. Cover'!C12</f>
+        <v/>
       </c>
     </row>
     <row r="23">
@@ -3913,7 +3935,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:H12"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -3926,7 +3948,19 @@
     <col width="16" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Blended EBITDA margin FY25A = 67.7%; Software revenue weight = 37.4%; Semi revenue weight = 62.6%</t>
+        </is>
+      </c>
+    </row>
     <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>If software EBITDA margin = 77% (Broadcom upper-bound), implied semi EBITDA margin = 62.0%</t>
+        </is>
+      </c>
       <c r="B2" s="18" t="inlineStr">
         <is>
           <t>SUM-OF-THE-PARTS (FY27E)</t>
@@ -4115,6 +4149,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 

</xml_diff>